<commit_message>
Add CoreWeave, Nebius, and IREN to Lease Matrix
Expanded the Lease Matrix sheet from 14 to 18 operators/providers with
neocloud rows highlighted in purple. Four sections now:

A. Operator × Tenant Matrix — 18 rows × 8 tenant columns (added CoreWeave,
   Nebius, IREN as both tenant columns AND as operator/provider rows)

B. Future Commitments — Added neocloud commitment data:
   - CoreWeave: $60.7B RPO, 1.9 GW capacity, sells to OpenAI/Meta/MSFT/Google
   - Nebius: ~$30B+ contracted, Meta $27B+$3B deals, MSFT multi-B, Nvidia $2B inv.
   - IREN: $9.7B Microsoft contract, 150K GPU target, owns all sites freehold

C. Top Customers by Operator — Added 3 neocloud rows plus Core Scientific

D. NEW: Neocloud Supply Chain Map — Detailed view of who each neocloud leases
   DC space from and who they sell compute to, with GPU fleets, Nvidia
   relationships, capacity figures, and 2026E ARR targets

Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/meta_leases_capex_analysis.xlsx
+++ b/meta_leases_capex_analysis.xlsx
@@ -25,7 +25,7 @@
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.00x"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -92,8 +92,19 @@
       <b val="1"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="004A235A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00999999"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -154,6 +165,18 @@
         <bgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2CCFF"/>
+        <bgColor rgb="00E2CCFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+        <bgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -201,7 +224,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -356,6 +379,31 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -721,25 +769,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J53"/>
+  <dimension ref="A1:K71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="48" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="50" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1">
+    <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Hyperscaler-to-Landlord Data Center Lease Matrix</t>
+          <t>Hyperscaler &amp; Neocloud Data Center Lease Matrix</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -751,11 +800,12 @@
       <c r="H1" s="1" t="n"/>
       <c r="I1" s="1" t="n"/>
       <c r="J1" s="1" t="n"/>
-    </row>
-    <row r="2" ht="20" customHeight="1">
+      <c r="K1" s="1" t="n"/>
+    </row>
+    <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Who leases from whom  |  Confirmed relationships as of Q1 2026  |  ✓ = confirmed tenant, ~ = suspected/indirect</t>
+          <t>Who leases from whom  |  Q1 2026 data  |  ✓ = confirmed tenant  |  ~ = suspected / indirect  |  Neoclouds highlighted in purple</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -767,12 +817,13 @@
       <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="n"/>
       <c r="J2" s="2" t="n"/>
-    </row>
-    <row r="3" ht="20" customHeight="1"/>
-    <row r="4" ht="20" customHeight="1">
+      <c r="K2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="22" customHeight="1"/>
+    <row r="4" ht="22" customHeight="1">
       <c r="A4" s="36" t="inlineStr">
         <is>
-          <t>A. DATA CENTER OPERATOR / LANDLORD  ×  HYPERSCALER TENANT MATRIX</t>
+          <t>A. DATA CENTER OPERATOR / LANDLORD  ×  TENANT MATRIX (Hyperscalers + Neoclouds)</t>
         </is>
       </c>
       <c r="B4" s="36" t="n"/>
@@ -784,8 +835,9 @@
       <c r="H4" s="36" t="n"/>
       <c r="I4" s="36" t="n"/>
       <c r="J4" s="36" t="n"/>
-    </row>
-    <row r="5" ht="20" customHeight="1">
+      <c r="K4" s="36" t="n"/>
+    </row>
+    <row r="5" ht="22" customHeight="1">
       <c r="A5" s="37" t="inlineStr">
         <is>
           <t>DC Operator / Landlord</t>
@@ -793,7 +845,7 @@
       </c>
       <c r="B5" s="37" t="inlineStr">
         <is>
-          <t>Capacity (GW)</t>
+          <t>Capacity</t>
         </is>
       </c>
       <c r="C5" s="37" t="inlineStr">
@@ -808,7 +860,7 @@
       </c>
       <c r="E5" s="37" t="inlineStr">
         <is>
-          <t>Google / Alphabet</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
@@ -823,24 +875,29 @@
       </c>
       <c r="H5" s="37" t="inlineStr">
         <is>
-          <t>CoreWeave / xAI</t>
+          <t>CoreWeave</t>
         </is>
       </c>
       <c r="I5" s="37" t="inlineStr">
         <is>
-          <t>Owner / Backer</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="J5" s="37" t="inlineStr">
         <is>
+          <t>IREN</t>
+        </is>
+      </c>
+      <c r="K5" s="37" t="inlineStr">
+        <is>
           <t>Key Notes</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="20" customHeight="1">
+    <row r="6" ht="22" customHeight="1">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>QTS Realty Trust</t>
+          <t>QTS Realty (Blackstone)</t>
         </is>
       </c>
       <c r="B6" s="38" t="inlineStr">
@@ -874,18 +931,15 @@
         </is>
       </c>
       <c r="H6" s="38" t="inlineStr"/>
-      <c r="I6" s="41" t="inlineStr">
-        <is>
-          <t>Blackstone ($10B acq. 2021)</t>
-        </is>
-      </c>
-      <c r="J6" s="41" t="inlineStr">
-        <is>
-          <t>Largest by MW; AWS anchor in ATL, CHI, NJ. $12B+ investment pipeline.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="20" customHeight="1">
+      <c r="I6" s="38" t="inlineStr"/>
+      <c r="J6" s="38" t="inlineStr"/>
+      <c r="K6" s="41" t="inlineStr">
+        <is>
+          <t>Largest by MW. AWS anchor ATL/CHI/NJ. $12B+ pipeline. Acquired for $10B (2021).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
       <c r="A7" s="42" t="inlineStr">
         <is>
           <t>Vantage Data Centers</t>
@@ -918,21 +972,18 @@
       </c>
       <c r="G7" s="43" t="inlineStr"/>
       <c r="H7" s="43" t="inlineStr"/>
-      <c r="I7" s="44" t="inlineStr">
-        <is>
-          <t>DigitalBridge / Silver Lake</t>
-        </is>
-      </c>
-      <c r="J7" s="44" t="inlineStr">
-        <is>
-          <t>100% hyperscale focus. Frontier Campus TX (1.4 GW), Port Washington WI (1.3 GW).</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="20" customHeight="1">
+      <c r="I7" s="43" t="inlineStr"/>
+      <c r="J7" s="43" t="inlineStr"/>
+      <c r="K7" s="44" t="inlineStr">
+        <is>
+          <t>100% hyperscale. Frontier TX (1.4 GW), Port Washington WI (1.3 GW). DigitalBridge/Silver Lake.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>Digital Realty Trust (DLR)</t>
+          <t>Digital Realty (DLR)</t>
         </is>
       </c>
       <c r="B8" s="38" t="inlineStr">
@@ -966,18 +1017,15 @@
         </is>
       </c>
       <c r="H8" s="38" t="inlineStr"/>
-      <c r="I8" s="41" t="inlineStr">
-        <is>
-          <t>Public REIT (NYSE: DLR)</t>
-        </is>
-      </c>
-      <c r="J8" s="41" t="inlineStr">
-        <is>
-          <t>310 DCs, 42.5M sq ft. $817M backlog. Broadest tenant diversification.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="20" customHeight="1">
+      <c r="I8" s="38" t="inlineStr"/>
+      <c r="J8" s="38" t="inlineStr"/>
+      <c r="K8" s="41" t="inlineStr">
+        <is>
+          <t>Public REIT. 310 DCs, 42.5M sq ft. $817M backlog. Broadest tenant diversification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
       <c r="A9" s="42" t="inlineStr">
         <is>
           <t>STACK Infrastructure</t>
@@ -1010,21 +1058,18 @@
         </is>
       </c>
       <c r="H9" s="43" t="inlineStr"/>
-      <c r="I9" s="44" t="inlineStr">
-        <is>
-          <t>IPI Partners / Mubadala</t>
-        </is>
-      </c>
-      <c r="J9" s="44" t="inlineStr">
-        <is>
-          <t>$12B Amazon partnership in Louisiana. 24 global markets. GW-scale campuses.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="20" customHeight="1">
+      <c r="I9" s="43" t="inlineStr"/>
+      <c r="J9" s="43" t="inlineStr"/>
+      <c r="K9" s="44" t="inlineStr">
+        <is>
+          <t>$12B Amazon partnership in Louisiana. IPI Partners / Mubadala. 24 global markets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>Aligned Data Centers</t>
+          <t>Aligned Data Centers (AIP)</t>
         </is>
       </c>
       <c r="B10" s="38" t="inlineStr">
@@ -1041,23 +1086,20 @@
       <c r="E10" s="38" t="inlineStr"/>
       <c r="F10" s="38" t="inlineStr"/>
       <c r="G10" s="38" t="inlineStr"/>
-      <c r="H10" s="39" t="inlineStr">
-        <is>
-          <t>✓ (xAI)</t>
-        </is>
-      </c>
-      <c r="I10" s="41" t="inlineStr">
-        <is>
-          <t>BlackRock AIP / Nvidia / MSFT / xAI</t>
-        </is>
-      </c>
-      <c r="J10" s="41" t="inlineStr">
-        <is>
-          <t>$40B acquisition (Oct 2025). 50 campuses. Largest DC deal in history.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="20" customHeight="1">
+      <c r="H10" s="38" t="inlineStr"/>
+      <c r="I10" s="38" t="inlineStr"/>
+      <c r="J10" s="39" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K10" s="41" t="inlineStr">
+        <is>
+          <t>$40B acq. by BlackRock/Nvidia/MSFT/xAI (Oct 2025). 50 campuses. Largest DC deal ever.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
       <c r="A11" s="42" t="inlineStr">
         <is>
           <t>Equinix (EQIX)</t>
@@ -1094,21 +1136,18 @@
         </is>
       </c>
       <c r="H11" s="43" t="inlineStr"/>
-      <c r="I11" s="44" t="inlineStr">
-        <is>
-          <t>Public REIT (NYSE: EQIX)</t>
-        </is>
-      </c>
-      <c r="J11" s="44" t="inlineStr">
-        <is>
-          <t>Interconnection-focused. 260+ DCs. 63% of Fortune 500. Direct cloud on-ramps.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
+      <c r="I11" s="43" t="inlineStr"/>
+      <c r="J11" s="43" t="inlineStr"/>
+      <c r="K11" s="44" t="inlineStr">
+        <is>
+          <t>Interconnection leader. 260+ DCs. 63% of F500. Low tenant concentration risk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>CyrusOne</t>
+          <t>CyrusOne (KKR/GIP)</t>
         </is>
       </c>
       <c r="B12" s="38" t="inlineStr">
@@ -1130,21 +1169,18 @@
       <c r="F12" s="38" t="inlineStr"/>
       <c r="G12" s="38" t="inlineStr"/>
       <c r="H12" s="38" t="inlineStr"/>
-      <c r="I12" s="41" t="inlineStr">
-        <is>
-          <t>KKR / GIP (acq. 2022)</t>
-        </is>
-      </c>
-      <c r="J12" s="41" t="inlineStr">
+      <c r="I12" s="38" t="inlineStr"/>
+      <c r="J12" s="38" t="inlineStr"/>
+      <c r="K12" s="41" t="inlineStr">
         <is>
           <t>AWS &amp; MSFT London leases. Calpine energy partnership (400 MW TX).</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="20" customHeight="1">
+    <row r="13" ht="22" customHeight="1">
       <c r="A13" s="42" t="inlineStr">
         <is>
-          <t>Compass Datacenters</t>
+          <t>Compass (Brookfield/OTPP)</t>
         </is>
       </c>
       <c r="B13" s="43" t="inlineStr">
@@ -1166,206 +1202,188 @@
       </c>
       <c r="G13" s="43" t="inlineStr"/>
       <c r="H13" s="43" t="inlineStr"/>
-      <c r="I13" s="44" t="inlineStr">
-        <is>
-          <t>Brookfield Infra / OTPP</t>
-        </is>
-      </c>
-      <c r="J13" s="44" t="inlineStr">
-        <is>
-          <t>$10B Meridian MS campus. Tenant undisclosed (suspected Meta or MSFT).</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="20" customHeight="1">
+      <c r="I13" s="43" t="inlineStr"/>
+      <c r="J13" s="43" t="inlineStr"/>
+      <c r="K13" s="44" t="inlineStr">
+        <is>
+          <t>$10B Meridian MS campus. Tenant undisclosed (suspected Meta or MSFT). Single-tenant modular.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>Crusoe Energy Systems</t>
+          <t>EdgeConneX (EQT)</t>
         </is>
       </c>
       <c r="B14" s="38" t="inlineStr">
         <is>
+          <t>1.0+ GW</t>
+        </is>
+      </c>
+      <c r="C14" s="39" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D14" s="39" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E14" s="39" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F14" s="40" t="inlineStr">
+        <is>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="G14" s="39" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H14" s="38" t="inlineStr"/>
+      <c r="I14" s="38" t="inlineStr"/>
+      <c r="J14" s="38" t="inlineStr"/>
+      <c r="K14" s="41" t="inlineStr">
+        <is>
+          <t>80+ DCs, 60+ markets, 20+ countries. Cloud on-ramps for all majors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="42" t="inlineStr">
+        <is>
+          <t>Crusoe Energy</t>
+        </is>
+      </c>
+      <c r="B15" s="43" t="inlineStr">
+        <is>
           <t>1.2 GW</t>
         </is>
       </c>
-      <c r="C14" s="38" t="inlineStr"/>
-      <c r="D14" s="40" t="inlineStr">
+      <c r="C15" s="43" t="inlineStr"/>
+      <c r="D15" s="40" t="inlineStr">
         <is>
           <t>~</t>
         </is>
       </c>
-      <c r="E14" s="38" t="inlineStr"/>
-      <c r="F14" s="38" t="inlineStr"/>
-      <c r="G14" s="39" t="inlineStr">
+      <c r="E15" s="43" t="inlineStr"/>
+      <c r="F15" s="43" t="inlineStr"/>
+      <c r="G15" s="39" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H14" s="38" t="inlineStr"/>
-      <c r="I14" s="41" t="inlineStr">
-        <is>
-          <t>Blue Owl / PE-backed</t>
-        </is>
-      </c>
-      <c r="J14" s="41" t="inlineStr">
-        <is>
-          <t>Abilene TX flagship. Oracle tenant → leases to MSFT → OpenAI. 15-yr lease.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="42" t="inlineStr">
-        <is>
-          <t>Hut 8 Corp</t>
-        </is>
-      </c>
-      <c r="B15" s="43" t="inlineStr">
+      <c r="H15" s="43" t="inlineStr"/>
+      <c r="I15" s="43" t="inlineStr"/>
+      <c r="J15" s="43" t="inlineStr"/>
+      <c r="K15" s="44" t="inlineStr">
+        <is>
+          <t>Abilene TX. Oracle tenant → MSFT → OpenAI sublease chain. Blue Owl JV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>Hut 8 Corp (HUT)</t>
+        </is>
+      </c>
+      <c r="B16" s="38" t="inlineStr">
         <is>
           <t>0.3 GW</t>
-        </is>
-      </c>
-      <c r="C15" s="43" t="inlineStr"/>
-      <c r="D15" s="43" t="inlineStr"/>
-      <c r="E15" s="39" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F15" s="43" t="inlineStr"/>
-      <c r="G15" s="43" t="inlineStr"/>
-      <c r="H15" s="43" t="inlineStr"/>
-      <c r="I15" s="44" t="inlineStr">
-        <is>
-          <t>Public (NASDAQ: HUT)</t>
-        </is>
-      </c>
-      <c r="J15" s="44" t="inlineStr">
-        <is>
-          <t>$7B, 15-yr lease w/ Fluidstack (Google-backed). River Bend LA. 245 MW.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="10" t="inlineStr">
-        <is>
-          <t>Applied Digital</t>
-        </is>
-      </c>
-      <c r="B16" s="38" t="inlineStr">
-        <is>
-          <t>0.4 GW</t>
         </is>
       </c>
       <c r="C16" s="38" t="inlineStr"/>
       <c r="D16" s="38" t="inlineStr"/>
-      <c r="E16" s="38" t="inlineStr"/>
+      <c r="E16" s="39" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="F16" s="38" t="inlineStr"/>
       <c r="G16" s="38" t="inlineStr"/>
-      <c r="H16" s="39" t="inlineStr">
-        <is>
-          <t>✓ (CoreWeave)</t>
-        </is>
-      </c>
-      <c r="I16" s="41" t="inlineStr">
-        <is>
-          <t>Public (NASDAQ: APLD)</t>
-        </is>
-      </c>
-      <c r="J16" s="41" t="inlineStr">
-        <is>
-          <t>$11B contracted from CoreWeave. Polaris Forge ND campus. 400 MW.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1">
+      <c r="H16" s="38" t="inlineStr"/>
+      <c r="I16" s="38" t="inlineStr"/>
+      <c r="J16" s="38" t="inlineStr"/>
+      <c r="K16" s="41" t="inlineStr">
+        <is>
+          <t>$7B/15-yr lease via Fluidstack (Google-backed). River Bend LA. 245 MW.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
       <c r="A17" s="42" t="inlineStr">
         <is>
-          <t>EdgeConneX</t>
+          <t>Applied Digital (APLD)</t>
         </is>
       </c>
       <c r="B17" s="43" t="inlineStr">
         <is>
-          <t>1.0+ GW</t>
-        </is>
-      </c>
-      <c r="C17" s="39" t="inlineStr">
+          <t>0.4 GW</t>
+        </is>
+      </c>
+      <c r="C17" s="43" t="inlineStr"/>
+      <c r="D17" s="43" t="inlineStr"/>
+      <c r="E17" s="43" t="inlineStr"/>
+      <c r="F17" s="43" t="inlineStr"/>
+      <c r="G17" s="43" t="inlineStr"/>
+      <c r="H17" s="39" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="D17" s="39" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E17" s="39" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F17" s="40" t="inlineStr">
-        <is>
-          <t>~</t>
-        </is>
-      </c>
-      <c r="G17" s="39" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H17" s="43" t="inlineStr"/>
-      <c r="I17" s="44" t="inlineStr">
-        <is>
-          <t>EQT Partners</t>
-        </is>
-      </c>
-      <c r="J17" s="44" t="inlineStr">
-        <is>
-          <t>80+ DCs, 60+ markets, 20+ countries. Cloud on-ramps for all major providers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1">
+      <c r="I17" s="43" t="inlineStr"/>
+      <c r="J17" s="43" t="inlineStr"/>
+      <c r="K17" s="44" t="inlineStr">
+        <is>
+          <t>$11B contracted from CoreWeave. Polaris Forge ND (400 MW). 15-yr triple-net leases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>Meta SPV (Pimco / Blue Owl)</t>
+          <t>Core Scientific (CORZ)</t>
         </is>
       </c>
       <c r="B18" s="38" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.3 GW</t>
         </is>
       </c>
       <c r="C18" s="38" t="inlineStr"/>
       <c r="D18" s="38" t="inlineStr"/>
       <c r="E18" s="38" t="inlineStr"/>
-      <c r="F18" s="39" t="inlineStr">
+      <c r="F18" s="38" t="inlineStr"/>
+      <c r="G18" s="38" t="inlineStr"/>
+      <c r="H18" s="39" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G18" s="38" t="inlineStr"/>
-      <c r="H18" s="38" t="inlineStr"/>
-      <c r="I18" s="41" t="inlineStr">
-        <is>
-          <t>Meta 20% co-ownership</t>
-        </is>
-      </c>
-      <c r="J18" s="41" t="inlineStr">
-        <is>
-          <t>Louisiana Hyperion: $29B Pimco debt + $3B Blue Owl equity. Build-to-suit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="20" customHeight="1">
+      <c r="I18" s="38" t="inlineStr"/>
+      <c r="J18" s="38" t="inlineStr"/>
+      <c r="K18" s="41" t="inlineStr">
+        <is>
+          <t>Acquired by CoreWeave for $9B (Jul 2025). 10 US sites. Pipeline to 2.3 GW.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
       <c r="A19" s="42" t="inlineStr">
         <is>
-          <t>Stargate JV (Oracle-led)</t>
+          <t>Stargate JV</t>
         </is>
       </c>
       <c r="B19" s="43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>4.5+ GW</t>
         </is>
       </c>
       <c r="C19" s="43" t="inlineStr"/>
@@ -1386,908 +1404,1720 @@
         </is>
       </c>
       <c r="H19" s="43" t="inlineStr"/>
-      <c r="I19" s="44" t="inlineStr">
-        <is>
-          <t>Oracle / SoftBank / OpenAI</t>
-        </is>
-      </c>
-      <c r="J19" s="44" t="inlineStr">
-        <is>
-          <t>Abilene TX mega-campus. MSFT &amp; Meta negotiating capacity. $500B vision.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="20" customHeight="1"/>
-    <row r="21" ht="20" customHeight="1"/>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="36" t="inlineStr">
-        <is>
-          <t>B. HYPERSCALER FUTURE LEASE COMMITMENTS (as of Q1 2026, $B)</t>
-        </is>
-      </c>
-      <c r="B22" s="36" t="n"/>
-      <c r="C22" s="36" t="n"/>
-      <c r="D22" s="36" t="n"/>
-      <c r="E22" s="36" t="n"/>
-      <c r="F22" s="36" t="n"/>
-      <c r="G22" s="36" t="n"/>
-      <c r="H22" s="36" t="n"/>
-      <c r="I22" s="36" t="n"/>
-      <c r="J22" s="36" t="n"/>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="45" t="inlineStr">
+      <c r="I19" s="43" t="inlineStr"/>
+      <c r="J19" s="43" t="inlineStr"/>
+      <c r="K19" s="44" t="inlineStr">
+        <is>
+          <t>Oracle/SoftBank/OpenAI. Abilene TX mega-campus. MSFT &amp; Meta negotiating capacity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>Meta SPV (Pimco/Blue Owl)</t>
+        </is>
+      </c>
+      <c r="B20" s="38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C20" s="38" t="inlineStr"/>
+      <c r="D20" s="38" t="inlineStr"/>
+      <c r="E20" s="38" t="inlineStr"/>
+      <c r="F20" s="39" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G20" s="38" t="inlineStr"/>
+      <c r="H20" s="38" t="inlineStr"/>
+      <c r="I20" s="38" t="inlineStr"/>
+      <c r="J20" s="38" t="inlineStr"/>
+      <c r="K20" s="41" t="inlineStr">
+        <is>
+          <t>Louisiana Hyperion: $26B Pimco debt + $3B Blue Owl equity. Meta 20% co-ownership.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="58" t="inlineStr">
+        <is>
+          <t>CoreWeave (CRWV)</t>
+        </is>
+      </c>
+      <c r="B21" s="59" t="inlineStr">
+        <is>
+          <t>1.9 GW</t>
+        </is>
+      </c>
+      <c r="C21" s="59" t="inlineStr"/>
+      <c r="D21" s="39" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E21" s="39" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F21" s="39" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G21" s="59" t="inlineStr"/>
+      <c r="H21" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I21" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J21" s="59" t="inlineStr"/>
+      <c r="K21" s="61" t="inlineStr">
+        <is>
+          <t>43 DCs. Sells GPU cloud to OpenAI ($22.4B), Meta ($14.2B), MSFT, Google. Nvidia-backed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="58" t="inlineStr">
+        <is>
+          <t>Nebius (NBIS)</t>
+        </is>
+      </c>
+      <c r="B22" s="59" t="inlineStr">
+        <is>
+          <t>0.2 GW</t>
+        </is>
+      </c>
+      <c r="C22" s="59" t="inlineStr"/>
+      <c r="D22" s="39" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E22" s="59" t="inlineStr"/>
+      <c r="F22" s="39" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G22" s="59" t="inlineStr"/>
+      <c r="H22" s="59" t="inlineStr"/>
+      <c r="I22" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J22" s="59" t="inlineStr"/>
+      <c r="K22" s="61" t="inlineStr">
+        <is>
+          <t>Meta ($27B+$3B deals), Microsoft (multi-B). Nvidia $2B investment. ARR $1.25B. Target 3 GW by end 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="58" t="inlineStr">
+        <is>
+          <t>IREN (formerly Iris Energy)</t>
+        </is>
+      </c>
+      <c r="B23" s="59" t="inlineStr">
+        <is>
+          <t>0.8 GW</t>
+        </is>
+      </c>
+      <c r="C23" s="59" t="inlineStr"/>
+      <c r="D23" s="39" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E23" s="59" t="inlineStr"/>
+      <c r="F23" s="59" t="inlineStr"/>
+      <c r="G23" s="59" t="inlineStr"/>
+      <c r="H23" s="59" t="inlineStr"/>
+      <c r="I23" s="59" t="inlineStr"/>
+      <c r="J23" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K23" s="61" t="inlineStr">
+        <is>
+          <t>MSFT $9.7B/5-yr contract. 150K GPU target. Childress TX 750 MW. Owns sites freehold.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1"/>
+    <row r="25" ht="22" customHeight="1"/>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="36" t="inlineStr">
+        <is>
+          <t>B. FUTURE LEASE &amp; CONTRACT COMMITMENTS — HYPERSCALERS + NEOCLOUDS (as of Q1 2026, $B)</t>
+        </is>
+      </c>
+      <c r="B26" s="36" t="n"/>
+      <c r="C26" s="36" t="n"/>
+      <c r="D26" s="36" t="n"/>
+      <c r="E26" s="36" t="n"/>
+      <c r="F26" s="36" t="n"/>
+      <c r="G26" s="36" t="n"/>
+      <c r="H26" s="36" t="n"/>
+      <c r="I26" s="36" t="n"/>
+      <c r="J26" s="36" t="n"/>
+      <c r="K26" s="36" t="n"/>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="45" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B27" s="37" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C27" s="37" t="inlineStr">
+        <is>
+          <t>Total Future Commitments ($B)</t>
+        </is>
+      </c>
+      <c r="D27" s="37" t="inlineStr">
+        <is>
+          <t>On-B/S Lease Liab. ($B)</t>
+        </is>
+      </c>
+      <c r="E27" s="37" t="inlineStr">
+        <is>
+          <t>Off-B/S / Uncommenced ($B)</t>
+        </is>
+      </c>
+      <c r="F27" s="37" t="inlineStr">
+        <is>
+          <t>2025 Revenue ($B)</t>
+        </is>
+      </c>
+      <c r="G27" s="37" t="inlineStr">
+        <is>
+          <t>Commit. / Revenue</t>
+        </is>
+      </c>
+      <c r="H27" s="37" t="inlineStr">
+        <is>
+          <t>Primary Strategy</t>
+        </is>
+      </c>
+      <c r="I27" s="37" t="inlineStr">
+        <is>
+          <t>Key Partners / Customers</t>
+        </is>
+      </c>
+      <c r="J27" s="46" t="inlineStr"/>
+      <c r="K27" s="46" t="inlineStr"/>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>Oracle</t>
+        </is>
+      </c>
+      <c r="B28" s="38" t="inlineStr">
         <is>
           <t>Hyperscaler</t>
         </is>
       </c>
-      <c r="B23" s="37" t="inlineStr">
-        <is>
-          <t>Total Future Lease Commitments ($B)</t>
-        </is>
-      </c>
-      <c r="C23" s="37" t="inlineStr">
-        <is>
-          <t>On-Balance-Sheet Lease Liab. ($B)</t>
-        </is>
-      </c>
-      <c r="D23" s="37" t="inlineStr">
-        <is>
-          <t>Off-B/S Uncommenced Leases ($B)</t>
-        </is>
-      </c>
-      <c r="E23" s="37" t="inlineStr">
-        <is>
-          <t>Lease Commit. / Revenue</t>
-        </is>
-      </c>
-      <c r="F23" s="37" t="inlineStr">
-        <is>
-          <t>Lease Commit. / Op. Income</t>
-        </is>
-      </c>
-      <c r="G23" s="37" t="inlineStr">
-        <is>
-          <t>Primary Lease Strategy</t>
-        </is>
-      </c>
-      <c r="H23" s="37" t="inlineStr">
-        <is>
-          <t>Key Landlord Partners</t>
-        </is>
-      </c>
-      <c r="I23" s="46" t="inlineStr"/>
-      <c r="J23" s="46" t="inlineStr"/>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="10" t="inlineStr">
+      <c r="C28" s="47" t="n">
+        <v>261</v>
+      </c>
+      <c r="D28" s="48" t="n">
+        <v>13</v>
+      </c>
+      <c r="E28" s="47" t="n">
+        <v>248</v>
+      </c>
+      <c r="F28" s="48" t="n">
+        <v>60</v>
+      </c>
+      <c r="G28" s="38" t="inlineStr">
+        <is>
+          <t>4.4x</t>
+        </is>
+      </c>
+      <c r="H28" s="41" t="inlineStr">
+        <is>
+          <t>Aggressive 3rd-party leasing; Stargate anchor</t>
+        </is>
+      </c>
+      <c r="I28" s="41" t="inlineStr">
+        <is>
+          <t>Crusoe, EdgeConneX, Stargate JV</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="42" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="B29" s="43" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="C29" s="50" t="n">
+        <v>155</v>
+      </c>
+      <c r="D29" s="50" t="n">
+        <v>50</v>
+      </c>
+      <c r="E29" s="50" t="n">
+        <v>105</v>
+      </c>
+      <c r="F29" s="50" t="n">
+        <v>281.7</v>
+      </c>
+      <c r="G29" s="43" t="inlineStr">
+        <is>
+          <t>0.6x</t>
+        </is>
+      </c>
+      <c r="H29" s="44" t="inlineStr">
+        <is>
+          <t>Mix owned + build-to-suit + co-invested (AIP)</t>
+        </is>
+      </c>
+      <c r="I29" s="44" t="inlineStr">
+        <is>
+          <t>Aligned, QTS, Vantage, CyrusOne, IREN, Nebius, CoreWeave</t>
+        </is>
+      </c>
+      <c r="J29" s="52" t="n"/>
+      <c r="K29" s="52" t="n"/>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="B30" s="38" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="C30" s="48" t="n">
+        <v>104</v>
+      </c>
+      <c r="D30" s="48" t="n">
+        <v>26.1</v>
+      </c>
+      <c r="E30" s="48" t="n">
+        <v>78</v>
+      </c>
+      <c r="F30" s="48" t="n">
+        <v>201</v>
+      </c>
+      <c r="G30" s="38" t="inlineStr">
+        <is>
+          <t>0.5x</t>
+        </is>
+      </c>
+      <c r="H30" s="41" t="inlineStr">
+        <is>
+          <t>SPV-financed build-to-suit; growing 3rd-party</t>
+        </is>
+      </c>
+      <c r="I30" s="41" t="inlineStr">
+        <is>
+          <t>Pimco/Blue Owl SPV, Digital Realty, Vantage, CoreWeave, Nebius</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="42" t="inlineStr">
+        <is>
+          <t>Google / Alphabet</t>
+        </is>
+      </c>
+      <c r="B31" s="43" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="C31" s="50" t="n">
+        <v>42.6</v>
+      </c>
+      <c r="D31" s="50" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="E31" s="50" t="n">
+        <v>20.1</v>
+      </c>
+      <c r="F31" s="50" t="n">
+        <v>402.8</v>
+      </c>
+      <c r="G31" s="43" t="inlineStr">
+        <is>
+          <t>0.1x</t>
+        </is>
+      </c>
+      <c r="H31" s="44" t="inlineStr">
+        <is>
+          <t>Mostly owned; selective leasing for speed</t>
+        </is>
+      </c>
+      <c r="I31" s="44" t="inlineStr">
+        <is>
+          <t>Hut 8 (Fluidstack), Digital Realty, Vantage, QTS, CoreWeave</t>
+        </is>
+      </c>
+      <c r="J31" s="52" t="n"/>
+      <c r="K31" s="52" t="n"/>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>Amazon / AWS</t>
+        </is>
+      </c>
+      <c r="B32" s="38" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="C32" s="38" t="inlineStr">
+        <is>
+          <t>~80–100</t>
+        </is>
+      </c>
+      <c r="D32" s="48" t="n">
+        <v>160</v>
+      </c>
+      <c r="E32" s="38" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F32" s="48" t="n">
+        <v>716.9</v>
+      </c>
+      <c r="G32" s="38" t="inlineStr">
+        <is>
+          <t>~0.1x</t>
+        </is>
+      </c>
+      <c r="H32" s="41" t="inlineStr">
+        <is>
+          <t>Mix owned mega-campuses + colocation at scale</t>
+        </is>
+      </c>
+      <c r="I32" s="41" t="inlineStr">
+        <is>
+          <t>QTS, STACK, Vantage, Digital Realty, EdgeConneX</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="62" t="inlineStr">
+        <is>
+          <t>CoreWeave</t>
+        </is>
+      </c>
+      <c r="B33" s="59" t="inlineStr">
+        <is>
+          <t>Neocloud</t>
+        </is>
+      </c>
+      <c r="C33" s="59" t="inlineStr">
+        <is>
+          <t>~60.7 (RPO)</t>
+        </is>
+      </c>
+      <c r="D33" s="59" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="E33" s="59" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F33" s="63" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="G33" s="59" t="inlineStr">
+        <is>
+          <t>~11.9x</t>
+        </is>
+      </c>
+      <c r="H33" s="61" t="inlineStr">
+        <is>
+          <t>Lease DCs → add GPUs → sell compute. Nvidia-backed</t>
+        </is>
+      </c>
+      <c r="I33" s="61" t="inlineStr">
+        <is>
+          <t>Tenants: Applied Digital, Core Scientific. Customers: OpenAI, Meta, MSFT, Google</t>
+        </is>
+      </c>
+      <c r="J33" s="64" t="n"/>
+      <c r="K33" s="64" t="n"/>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="62" t="inlineStr">
+        <is>
+          <t>Nebius</t>
+        </is>
+      </c>
+      <c r="B34" s="59" t="inlineStr">
+        <is>
+          <t>Neocloud</t>
+        </is>
+      </c>
+      <c r="C34" s="59" t="inlineStr">
+        <is>
+          <t>~30+ (contracted)</t>
+        </is>
+      </c>
+      <c r="D34" s="59" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="E34" s="59" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F34" s="63" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="G34" s="59" t="inlineStr">
+        <is>
+          <t>~57x</t>
+        </is>
+      </c>
+      <c r="H34" s="61" t="inlineStr">
+        <is>
+          <t>Build-to-own + colocation. Nvidia $2B investment</t>
+        </is>
+      </c>
+      <c r="I34" s="61" t="inlineStr">
+        <is>
+          <t>Customers: Meta ($27B+$3B), Microsoft. Landlords: Patmos (KC). Mostly self-built</t>
+        </is>
+      </c>
+      <c r="J34" s="64" t="n"/>
+      <c r="K34" s="64" t="n"/>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="62" t="inlineStr">
+        <is>
+          <t>IREN</t>
+        </is>
+      </c>
+      <c r="B35" s="59" t="inlineStr">
+        <is>
+          <t>Neocloud</t>
+        </is>
+      </c>
+      <c r="C35" s="59" t="inlineStr">
+        <is>
+          <t>~9.7 (MSFT contract)</t>
+        </is>
+      </c>
+      <c r="D35" s="59" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="E35" s="59" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F35" s="63" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="G35" s="59" t="inlineStr">
+        <is>
+          <t>~10x</t>
+        </is>
+      </c>
+      <c r="H35" s="61" t="inlineStr">
+        <is>
+          <t>Owner-operator. Freehold sites. GPU-as-a-service</t>
+        </is>
+      </c>
+      <c r="I35" s="61" t="inlineStr">
+        <is>
+          <t>Customers: Microsoft ($9.7B), Together AI, Fluidstack, Fireworks AI</t>
+        </is>
+      </c>
+      <c r="J35" s="64" t="n"/>
+      <c r="K35" s="64" t="n"/>
+    </row>
+    <row r="36" ht="22" customHeight="1"/>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="36" t="inlineStr">
+        <is>
+          <t>C. TOP CUSTOMERS / TENANTS BY OPERATOR (Ranked by Estimated Revenue Contribution)</t>
+        </is>
+      </c>
+      <c r="B37" s="36" t="n"/>
+      <c r="C37" s="36" t="n"/>
+      <c r="D37" s="36" t="n"/>
+      <c r="E37" s="36" t="n"/>
+      <c r="F37" s="36" t="n"/>
+      <c r="G37" s="36" t="n"/>
+      <c r="H37" s="36" t="n"/>
+      <c r="I37" s="36" t="n"/>
+      <c r="J37" s="36" t="n"/>
+      <c r="K37" s="36" t="n"/>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="45" t="inlineStr">
+        <is>
+          <t>DC Operator / Provider</t>
+        </is>
+      </c>
+      <c r="B38" s="37" t="inlineStr">
+        <is>
+          <t>#1 Customer</t>
+        </is>
+      </c>
+      <c r="C38" s="37" t="inlineStr">
+        <is>
+          <t>#2 Customer</t>
+        </is>
+      </c>
+      <c r="D38" s="37" t="inlineStr">
+        <is>
+          <t>#3 Customer</t>
+        </is>
+      </c>
+      <c r="E38" s="37" t="inlineStr">
+        <is>
+          <t>Concentration Risk</t>
+        </is>
+      </c>
+      <c r="F38" s="37" t="inlineStr">
+        <is>
+          <t>Avg Lease Term</t>
+        </is>
+      </c>
+      <c r="G38" s="37" t="inlineStr">
+        <is>
+          <t>Lease / Contract Structure</t>
+        </is>
+      </c>
+      <c r="H38" s="37" t="inlineStr">
+        <is>
+          <t>Est. Annual Rev from Top 3 ($B)</t>
+        </is>
+      </c>
+      <c r="I38" s="37" t="inlineStr">
+        <is>
+          <t>Owner / Backer</t>
+        </is>
+      </c>
+      <c r="J38" s="46" t="inlineStr"/>
+      <c r="K38" s="46" t="inlineStr"/>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t>QTS (Blackstone)</t>
+        </is>
+      </c>
+      <c r="B39" s="38" t="inlineStr">
+        <is>
+          <t>Amazon / AWS</t>
+        </is>
+      </c>
+      <c r="C39" s="38" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="D39" s="38" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="E39" s="53" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F39" s="38" t="inlineStr">
+        <is>
+          <t>10–20 yrs</t>
+        </is>
+      </c>
+      <c r="G39" s="41" t="inlineStr">
+        <is>
+          <t>Triple-net, build-to-suit</t>
+        </is>
+      </c>
+      <c r="H39" s="38" t="inlineStr">
+        <is>
+          <t>$4–6</t>
+        </is>
+      </c>
+      <c r="I39" s="41" t="inlineStr">
+        <is>
+          <t>Blackstone ($10B acq.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="42" t="inlineStr">
+        <is>
+          <t>Vantage</t>
+        </is>
+      </c>
+      <c r="B40" s="43" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="C40" s="43" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="D40" s="43" t="inlineStr">
+        <is>
+          <t>Amazon / AWS</t>
+        </is>
+      </c>
+      <c r="E40" s="54" t="inlineStr">
+        <is>
+          <t>Very High</t>
+        </is>
+      </c>
+      <c r="F40" s="43" t="inlineStr">
+        <is>
+          <t>15–20 yrs</t>
+        </is>
+      </c>
+      <c r="G40" s="44" t="inlineStr">
+        <is>
+          <t>Single-tenant, shell + core</t>
+        </is>
+      </c>
+      <c r="H40" s="43" t="inlineStr">
+        <is>
+          <t>$3–5</t>
+        </is>
+      </c>
+      <c r="I40" s="44" t="inlineStr">
+        <is>
+          <t>DigitalBridge / Silver Lake</t>
+        </is>
+      </c>
+      <c r="J40" s="52" t="n"/>
+      <c r="K40" s="52" t="n"/>
+    </row>
+    <row r="41" ht="22" customHeight="1">
+      <c r="A41" s="10" t="inlineStr">
+        <is>
+          <t>Digital Realty (DLR)</t>
+        </is>
+      </c>
+      <c r="B41" s="38" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="C41" s="38" t="inlineStr">
         <is>
           <t>Oracle</t>
         </is>
       </c>
-      <c r="B24" s="47" t="n">
-        <v>261</v>
-      </c>
-      <c r="C24" s="48" t="n">
-        <v>13</v>
-      </c>
-      <c r="D24" s="47" t="n">
-        <v>248</v>
-      </c>
-      <c r="E24" s="49" t="n">
-        <v>4.35</v>
-      </c>
-      <c r="F24" s="49" t="n">
-        <v>14.5</v>
-      </c>
-      <c r="G24" s="41" t="inlineStr">
-        <is>
-          <t>Aggressive third-party leasing; Stargate anchor</t>
-        </is>
-      </c>
-      <c r="H24" s="41" t="inlineStr">
-        <is>
-          <t>Crusoe, Stargate JV, EdgeConneX</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="42" t="inlineStr">
+      <c r="D41" s="38" t="inlineStr">
+        <is>
+          <t>Amazon / AWS</t>
+        </is>
+      </c>
+      <c r="E41" s="41" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="F41" s="38" t="inlineStr">
+        <is>
+          <t>7–15 yrs</t>
+        </is>
+      </c>
+      <c r="G41" s="41" t="inlineStr">
+        <is>
+          <t>Mix: colo + build-to-suit</t>
+        </is>
+      </c>
+      <c r="H41" s="38" t="inlineStr">
+        <is>
+          <t>$2–4</t>
+        </is>
+      </c>
+      <c r="I41" s="41" t="inlineStr">
+        <is>
+          <t>Public REIT (NYSE: DLR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="22" customHeight="1">
+      <c r="A42" s="42" t="inlineStr">
+        <is>
+          <t>STACK Infrastructure</t>
+        </is>
+      </c>
+      <c r="B42" s="43" t="inlineStr">
+        <is>
+          <t>Amazon / AWS</t>
+        </is>
+      </c>
+      <c r="C42" s="43" t="inlineStr">
+        <is>
+          <t>Oracle</t>
+        </is>
+      </c>
+      <c r="D42" s="43" t="inlineStr">
         <is>
           <t>Microsoft</t>
         </is>
       </c>
-      <c r="B25" s="50" t="n">
-        <v>155</v>
-      </c>
-      <c r="C25" s="50" t="n">
-        <v>50</v>
-      </c>
-      <c r="D25" s="50" t="n">
-        <v>105</v>
-      </c>
-      <c r="E25" s="51" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F25" s="51" t="n">
-        <v>1.21</v>
-      </c>
-      <c r="G25" s="44" t="inlineStr">
-        <is>
-          <t>Mix of owned + build-to-suit + co-invested (AIP/Aligned)</t>
-        </is>
-      </c>
-      <c r="H25" s="44" t="inlineStr">
-        <is>
-          <t>Aligned, QTS, Vantage, CyrusOne, Compass</t>
-        </is>
-      </c>
-      <c r="I25" s="52" t="n"/>
-      <c r="J25" s="52" t="n"/>
-    </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
-      <c r="B26" s="48" t="n">
-        <v>104</v>
-      </c>
-      <c r="C26" s="48" t="n">
-        <v>26.1</v>
-      </c>
-      <c r="D26" s="48" t="n">
-        <v>78</v>
-      </c>
-      <c r="E26" s="49" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="F26" s="49" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="G26" s="41" t="inlineStr">
-        <is>
-          <t>SPV-financed build-to-suit; growing third-party leasing</t>
-        </is>
-      </c>
-      <c r="H26" s="41" t="inlineStr">
-        <is>
-          <t>Pimco/Blue Owl SPV, Digital Realty, Vantage, EdgeConneX</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="42" t="inlineStr">
-        <is>
-          <t>Google / Alphabet</t>
-        </is>
-      </c>
-      <c r="B27" s="50" t="n">
-        <v>42.6</v>
-      </c>
-      <c r="C27" s="50" t="n">
-        <v>22.5</v>
-      </c>
-      <c r="D27" s="50" t="n">
-        <v>20.1</v>
-      </c>
-      <c r="E27" s="51" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="F27" s="51" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="G27" s="44" t="inlineStr">
-        <is>
-          <t>Mostly owned; selective leasing for speed-to-capacity</t>
-        </is>
-      </c>
-      <c r="H27" s="44" t="inlineStr">
-        <is>
-          <t>Hut 8 (Fluidstack), Digital Realty, Vantage, QTS</t>
-        </is>
-      </c>
-      <c r="I27" s="52" t="n"/>
-      <c r="J27" s="52" t="n"/>
-    </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="10" t="inlineStr">
+      <c r="E42" s="53" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F42" s="43" t="inlineStr">
+        <is>
+          <t>15–25 yrs</t>
+        </is>
+      </c>
+      <c r="G42" s="44" t="inlineStr">
+        <is>
+          <t>Powered shell, triple-net</t>
+        </is>
+      </c>
+      <c r="H42" s="43" t="inlineStr">
+        <is>
+          <t>$2–3</t>
+        </is>
+      </c>
+      <c r="I42" s="44" t="inlineStr">
+        <is>
+          <t>IPI Partners / Mubadala</t>
+        </is>
+      </c>
+      <c r="J42" s="52" t="n"/>
+      <c r="K42" s="52" t="n"/>
+    </row>
+    <row r="43" ht="22" customHeight="1">
+      <c r="A43" s="10" t="inlineStr">
+        <is>
+          <t>Aligned (BlackRock AIP)</t>
+        </is>
+      </c>
+      <c r="B43" s="38" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="C43" s="38" t="inlineStr">
+        <is>
+          <t>xAI</t>
+        </is>
+      </c>
+      <c r="D43" s="38" t="inlineStr">
+        <is>
+          <t>IREN</t>
+        </is>
+      </c>
+      <c r="E43" s="54" t="inlineStr">
+        <is>
+          <t>Very High</t>
+        </is>
+      </c>
+      <c r="F43" s="38" t="inlineStr">
+        <is>
+          <t>10–20 yrs</t>
+        </is>
+      </c>
+      <c r="G43" s="41" t="inlineStr">
+        <is>
+          <t>Co-invested, build-to-suit</t>
+        </is>
+      </c>
+      <c r="H43" s="38" t="inlineStr">
+        <is>
+          <t>$2–4</t>
+        </is>
+      </c>
+      <c r="I43" s="41" t="inlineStr">
+        <is>
+          <t>BlackRock / Nvidia / MSFT / xAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="42" t="inlineStr">
+        <is>
+          <t>Equinix (EQIX)</t>
+        </is>
+      </c>
+      <c r="B44" s="43" t="inlineStr">
         <is>
           <t>Amazon / AWS</t>
         </is>
       </c>
-      <c r="B28" s="38" t="inlineStr">
-        <is>
-          <t>~80-100</t>
-        </is>
-      </c>
-      <c r="C28" s="48" t="n">
-        <v>160</v>
-      </c>
-      <c r="D28" s="38" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="E28" s="38" t="inlineStr">
-        <is>
-          <t>~0.13</t>
-        </is>
-      </c>
-      <c r="F28" s="38" t="inlineStr">
-        <is>
-          <t>~1.2</t>
-        </is>
-      </c>
-      <c r="G28" s="41" t="inlineStr">
-        <is>
-          <t>Mix of owned mega-campuses + colocation at scale</t>
-        </is>
-      </c>
-      <c r="H28" s="41" t="inlineStr">
-        <is>
-          <t>QTS, STACK, Vantage, Digital Realty, EdgeConneX</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="20" customHeight="1"/>
-    <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="36" t="inlineStr">
-        <is>
-          <t>C. TOP CUSTOMERS / TENANTS BY DATA CENTER OPERATOR (Ranked by Estimated Revenue Contribution)</t>
-        </is>
-      </c>
-      <c r="B30" s="36" t="n"/>
-      <c r="C30" s="36" t="n"/>
-      <c r="D30" s="36" t="n"/>
-      <c r="E30" s="36" t="n"/>
-      <c r="F30" s="36" t="n"/>
-      <c r="G30" s="36" t="n"/>
-      <c r="H30" s="36" t="n"/>
-      <c r="I30" s="36" t="n"/>
-      <c r="J30" s="36" t="n"/>
-    </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="37" t="inlineStr">
-        <is>
-          <t>DC Operator</t>
-        </is>
-      </c>
-      <c r="B31" s="37" t="inlineStr">
-        <is>
-          <t>#1 Customer</t>
-        </is>
-      </c>
-      <c r="C31" s="37" t="inlineStr">
-        <is>
-          <t>#2 Customer</t>
-        </is>
-      </c>
-      <c r="D31" s="37" t="inlineStr">
-        <is>
-          <t>#3 Customer</t>
-        </is>
-      </c>
-      <c r="E31" s="37" t="inlineStr">
-        <is>
-          <t>Revenue Concentration Risk</t>
-        </is>
-      </c>
-      <c r="F31" s="37" t="inlineStr">
-        <is>
-          <t>Avg Lease Term (Yrs)</t>
-        </is>
-      </c>
-      <c r="G31" s="37" t="inlineStr">
-        <is>
-          <t>Lease Structure</t>
-        </is>
-      </c>
-      <c r="H31" s="37" t="inlineStr">
-        <is>
-          <t>Est. Annual Rent from Top 3 ($B)</t>
-        </is>
-      </c>
-      <c r="I31" s="46" t="inlineStr"/>
-      <c r="J31" s="46" t="inlineStr"/>
-    </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="10" t="inlineStr">
-        <is>
-          <t>QTS (Blackstone)</t>
-        </is>
-      </c>
-      <c r="B32" s="38" t="inlineStr">
+      <c r="C44" s="43" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="D44" s="43" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="E44" s="65" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F44" s="43" t="inlineStr">
+        <is>
+          <t>3–5 yrs</t>
+        </is>
+      </c>
+      <c r="G44" s="44" t="inlineStr">
+        <is>
+          <t>Retail colo + interconnection</t>
+        </is>
+      </c>
+      <c r="H44" s="43" t="inlineStr">
+        <is>
+          <t>$1–2</t>
+        </is>
+      </c>
+      <c r="I44" s="44" t="inlineStr">
+        <is>
+          <t>Public REIT (NYSE: EQIX)</t>
+        </is>
+      </c>
+      <c r="J44" s="52" t="n"/>
+      <c r="K44" s="52" t="n"/>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="10" t="inlineStr">
+        <is>
+          <t>CyrusOne (KKR/GIP)</t>
+        </is>
+      </c>
+      <c r="B45" s="38" t="inlineStr">
         <is>
           <t>Amazon / AWS</t>
         </is>
       </c>
-      <c r="C32" s="38" t="inlineStr">
+      <c r="C45" s="38" t="inlineStr">
         <is>
           <t>Microsoft</t>
         </is>
       </c>
-      <c r="D32" s="38" t="inlineStr">
-        <is>
-          <t>Google</t>
-        </is>
-      </c>
-      <c r="E32" s="53" t="inlineStr">
-        <is>
-          <t>High — dominated by 2-3 hyperscalers</t>
-        </is>
-      </c>
-      <c r="F32" s="38" t="inlineStr">
-        <is>
-          <t>10-20</t>
-        </is>
-      </c>
-      <c r="G32" s="41" t="inlineStr">
-        <is>
-          <t>Triple-net, build-to-suit</t>
-        </is>
-      </c>
-      <c r="H32" s="38" t="inlineStr">
-        <is>
-          <t>~$4-6</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="42" t="inlineStr">
-        <is>
-          <t>Vantage</t>
-        </is>
-      </c>
-      <c r="B33" s="43" t="inlineStr">
+      <c r="D45" s="38" t="inlineStr">
+        <is>
+          <t>Enterprise mix</t>
+        </is>
+      </c>
+      <c r="E45" s="41" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="F45" s="38" t="inlineStr">
+        <is>
+          <t>10–15 yrs</t>
+        </is>
+      </c>
+      <c r="G45" s="41" t="inlineStr">
+        <is>
+          <t>Build-to-suit hyperscale</t>
+        </is>
+      </c>
+      <c r="H45" s="38" t="inlineStr">
+        <is>
+          <t>$0.5–1</t>
+        </is>
+      </c>
+      <c r="I45" s="41" t="inlineStr">
+        <is>
+          <t>KKR / GIP</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="42" t="inlineStr">
+        <is>
+          <t>Compass (Brookfield)</t>
+        </is>
+      </c>
+      <c r="B46" s="43" t="inlineStr">
+        <is>
+          <t>Undisclosed (Meta or MSFT)</t>
+        </is>
+      </c>
+      <c r="C46" s="43" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D46" s="43" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E46" s="54" t="inlineStr">
+        <is>
+          <t>Very High</t>
+        </is>
+      </c>
+      <c r="F46" s="43" t="inlineStr">
+        <is>
+          <t>15–20 yrs</t>
+        </is>
+      </c>
+      <c r="G46" s="44" t="inlineStr">
+        <is>
+          <t>Single-tenant modular</t>
+        </is>
+      </c>
+      <c r="H46" s="43" t="inlineStr">
+        <is>
+          <t>$1–2</t>
+        </is>
+      </c>
+      <c r="I46" s="44" t="inlineStr">
+        <is>
+          <t>Brookfield Infra / OTPP</t>
+        </is>
+      </c>
+      <c r="J46" s="52" t="n"/>
+      <c r="K46" s="52" t="n"/>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="10" t="inlineStr">
+        <is>
+          <t>Crusoe Energy</t>
+        </is>
+      </c>
+      <c r="B47" s="38" t="inlineStr">
+        <is>
+          <t>Oracle</t>
+        </is>
+      </c>
+      <c r="C47" s="38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D47" s="38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E47" s="55" t="inlineStr">
+        <is>
+          <t>Extreme</t>
+        </is>
+      </c>
+      <c r="F47" s="38" t="inlineStr">
+        <is>
+          <t>15 yrs</t>
+        </is>
+      </c>
+      <c r="G47" s="41" t="inlineStr">
+        <is>
+          <t>Build-to-suit, triple-net</t>
+        </is>
+      </c>
+      <c r="H47" s="38" t="inlineStr">
+        <is>
+          <t>$1–2</t>
+        </is>
+      </c>
+      <c r="I47" s="41" t="inlineStr">
+        <is>
+          <t>Blue Owl / PE-backed</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="42" t="inlineStr">
+        <is>
+          <t>Hut 8 (HUT)</t>
+        </is>
+      </c>
+      <c r="B48" s="43" t="inlineStr">
+        <is>
+          <t>Google (via Fluidstack)</t>
+        </is>
+      </c>
+      <c r="C48" s="43" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D48" s="43" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E48" s="55" t="inlineStr">
+        <is>
+          <t>Extreme</t>
+        </is>
+      </c>
+      <c r="F48" s="43" t="inlineStr">
+        <is>
+          <t>15 (+15 renewal)</t>
+        </is>
+      </c>
+      <c r="G48" s="44" t="inlineStr">
+        <is>
+          <t>Triple-net IT lease</t>
+        </is>
+      </c>
+      <c r="H48" s="43" t="inlineStr">
+        <is>
+          <t>$0.5</t>
+        </is>
+      </c>
+      <c r="I48" s="44" t="inlineStr">
+        <is>
+          <t>Public (NASDAQ: HUT)</t>
+        </is>
+      </c>
+      <c r="J48" s="52" t="n"/>
+      <c r="K48" s="52" t="n"/>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="10" t="inlineStr">
+        <is>
+          <t>Applied Digital (APLD)</t>
+        </is>
+      </c>
+      <c r="B49" s="38" t="inlineStr">
+        <is>
+          <t>CoreWeave</t>
+        </is>
+      </c>
+      <c r="C49" s="38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D49" s="38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E49" s="55" t="inlineStr">
+        <is>
+          <t>Extreme</t>
+        </is>
+      </c>
+      <c r="F49" s="38" t="inlineStr">
+        <is>
+          <t>15 yrs</t>
+        </is>
+      </c>
+      <c r="G49" s="41" t="inlineStr">
+        <is>
+          <t>Triple-net, GPU-ready shell</t>
+        </is>
+      </c>
+      <c r="H49" s="38" t="inlineStr">
+        <is>
+          <t>$0.7</t>
+        </is>
+      </c>
+      <c r="I49" s="41" t="inlineStr">
+        <is>
+          <t>Public (NASDAQ: APLD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="42" t="inlineStr">
+        <is>
+          <t>Core Scientific (CORZ)</t>
+        </is>
+      </c>
+      <c r="B50" s="43" t="inlineStr">
+        <is>
+          <t>CoreWeave</t>
+        </is>
+      </c>
+      <c r="C50" s="43" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D50" s="43" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E50" s="55" t="inlineStr">
+        <is>
+          <t>Extreme</t>
+        </is>
+      </c>
+      <c r="F50" s="43" t="inlineStr">
+        <is>
+          <t>12–15 yrs</t>
+        </is>
+      </c>
+      <c r="G50" s="44" t="inlineStr">
+        <is>
+          <t>Acquired by CoreWeave ($9B)</t>
+        </is>
+      </c>
+      <c r="H50" s="43" t="inlineStr">
+        <is>
+          <t>$0.5–1</t>
+        </is>
+      </c>
+      <c r="I50" s="44" t="inlineStr">
+        <is>
+          <t>CoreWeave (acquired Jul 2025)</t>
+        </is>
+      </c>
+      <c r="J50" s="52" t="n"/>
+      <c r="K50" s="52" t="n"/>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="10" t="inlineStr">
+        <is>
+          <t>EdgeConneX (EQT)</t>
+        </is>
+      </c>
+      <c r="B51" s="38" t="inlineStr">
+        <is>
+          <t>Mixed hyperscale</t>
+        </is>
+      </c>
+      <c r="C51" s="38" t="inlineStr">
+        <is>
+          <t>Oracle</t>
+        </is>
+      </c>
+      <c r="D51" s="38" t="inlineStr">
+        <is>
+          <t>AWS / MSFT</t>
+        </is>
+      </c>
+      <c r="E51" s="41" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="F51" s="38" t="inlineStr">
+        <is>
+          <t>10–15 yrs</t>
+        </is>
+      </c>
+      <c r="G51" s="41" t="inlineStr">
+        <is>
+          <t>Build-to-suit colo</t>
+        </is>
+      </c>
+      <c r="H51" s="38" t="inlineStr">
+        <is>
+          <t>$0.5–1</t>
+        </is>
+      </c>
+      <c r="I51" s="41" t="inlineStr">
+        <is>
+          <t>EQT Partners</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="A52" s="62" t="inlineStr">
+        <is>
+          <t>CoreWeave (CRWV)</t>
+        </is>
+      </c>
+      <c r="B52" s="59" t="inlineStr">
+        <is>
+          <t>OpenAI ($22.4B)</t>
+        </is>
+      </c>
+      <c r="C52" s="59" t="inlineStr">
+        <is>
+          <t>Meta ($14.2B)</t>
+        </is>
+      </c>
+      <c r="D52" s="59" t="inlineStr">
         <is>
           <t>Microsoft</t>
         </is>
       </c>
-      <c r="C33" s="43" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
-      <c r="D33" s="43" t="inlineStr">
-        <is>
-          <t>Amazon / AWS</t>
-        </is>
-      </c>
-      <c r="E33" s="54" t="inlineStr">
-        <is>
-          <t>Very High — 100% hyperscale</t>
-        </is>
-      </c>
-      <c r="F33" s="43" t="inlineStr">
-        <is>
-          <t>15-20</t>
-        </is>
-      </c>
-      <c r="G33" s="44" t="inlineStr">
-        <is>
-          <t>Single-tenant, shell + core</t>
-        </is>
-      </c>
-      <c r="H33" s="43" t="inlineStr">
-        <is>
-          <t>~$3-5</t>
-        </is>
-      </c>
-      <c r="I33" s="52" t="n"/>
-      <c r="J33" s="52" t="n"/>
-    </row>
-    <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="10" t="inlineStr">
-        <is>
-          <t>Digital Realty (DLR)</t>
-        </is>
-      </c>
-      <c r="B34" s="38" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
-      <c r="C34" s="38" t="inlineStr">
-        <is>
-          <t>Oracle</t>
-        </is>
-      </c>
-      <c r="D34" s="38" t="inlineStr">
-        <is>
-          <t>Amazon / AWS</t>
-        </is>
-      </c>
-      <c r="E34" s="41" t="inlineStr">
-        <is>
-          <t>Moderate — diversified portfolio</t>
-        </is>
-      </c>
-      <c r="F34" s="38" t="inlineStr">
-        <is>
-          <t>7-15</t>
-        </is>
-      </c>
-      <c r="G34" s="41" t="inlineStr">
-        <is>
-          <t>Mix: colo + build-to-suit</t>
-        </is>
-      </c>
-      <c r="H34" s="38" t="inlineStr">
-        <is>
-          <t>~$2-4</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="42" t="inlineStr">
-        <is>
-          <t>STACK Infrastructure</t>
-        </is>
-      </c>
-      <c r="B35" s="43" t="inlineStr">
-        <is>
-          <t>Amazon / AWS</t>
-        </is>
-      </c>
-      <c r="C35" s="43" t="inlineStr">
-        <is>
-          <t>Oracle</t>
-        </is>
-      </c>
-      <c r="D35" s="43" t="inlineStr">
-        <is>
-          <t>Microsoft</t>
-        </is>
-      </c>
-      <c r="E35" s="53" t="inlineStr">
-        <is>
-          <t>High — anchor-tenant campuses</t>
-        </is>
-      </c>
-      <c r="F35" s="43" t="inlineStr">
-        <is>
-          <t>15-25</t>
-        </is>
-      </c>
-      <c r="G35" s="44" t="inlineStr">
-        <is>
-          <t>Powered shell, triple-net</t>
-        </is>
-      </c>
-      <c r="H35" s="43" t="inlineStr">
-        <is>
-          <t>~$2-3</t>
-        </is>
-      </c>
-      <c r="I35" s="52" t="n"/>
-      <c r="J35" s="52" t="n"/>
-    </row>
-    <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="10" t="inlineStr">
-        <is>
-          <t>Aligned (BlackRock AIP)</t>
-        </is>
-      </c>
-      <c r="B36" s="38" t="inlineStr">
-        <is>
-          <t>Microsoft</t>
-        </is>
-      </c>
-      <c r="C36" s="38" t="inlineStr">
-        <is>
-          <t>xAI</t>
-        </is>
-      </c>
-      <c r="D36" s="38" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E36" s="54" t="inlineStr">
-        <is>
-          <t>Very High — consortium-owned</t>
-        </is>
-      </c>
-      <c r="F36" s="38" t="inlineStr">
-        <is>
-          <t>10-20</t>
-        </is>
-      </c>
-      <c r="G36" s="41" t="inlineStr">
-        <is>
-          <t>Co-invested, build-to-suit</t>
-        </is>
-      </c>
-      <c r="H36" s="38" t="inlineStr">
-        <is>
-          <t>~$2-4</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="42" t="inlineStr">
-        <is>
-          <t>Equinix (EQIX)</t>
-        </is>
-      </c>
-      <c r="B37" s="43" t="inlineStr">
-        <is>
-          <t>Amazon / AWS</t>
-        </is>
-      </c>
-      <c r="C37" s="43" t="inlineStr">
-        <is>
-          <t>Microsoft</t>
-        </is>
-      </c>
-      <c r="D37" s="43" t="inlineStr">
-        <is>
-          <t>Google</t>
-        </is>
-      </c>
-      <c r="E37" s="53" t="inlineStr">
-        <is>
-          <t>Low — highly diversified (10K+ customers)</t>
-        </is>
-      </c>
-      <c r="F37" s="43" t="inlineStr">
-        <is>
-          <t>3-5</t>
-        </is>
-      </c>
-      <c r="G37" s="44" t="inlineStr">
-        <is>
-          <t>Retail colo + interconnection</t>
-        </is>
-      </c>
-      <c r="H37" s="43" t="inlineStr">
-        <is>
-          <t>~$1-2</t>
-        </is>
-      </c>
-      <c r="I37" s="52" t="n"/>
-      <c r="J37" s="52" t="n"/>
-    </row>
-    <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="10" t="inlineStr">
-        <is>
-          <t>CyrusOne (KKR/GIP)</t>
-        </is>
-      </c>
-      <c r="B38" s="38" t="inlineStr">
-        <is>
-          <t>Amazon / AWS</t>
-        </is>
-      </c>
-      <c r="C38" s="38" t="inlineStr">
-        <is>
-          <t>Microsoft</t>
-        </is>
-      </c>
-      <c r="D38" s="38" t="inlineStr">
-        <is>
-          <t>Enterprise mix</t>
-        </is>
-      </c>
-      <c r="E38" s="41" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-      <c r="F38" s="38" t="inlineStr">
-        <is>
-          <t>10-15</t>
-        </is>
-      </c>
-      <c r="G38" s="41" t="inlineStr">
-        <is>
-          <t>Build-to-suit hyperscale</t>
-        </is>
-      </c>
-      <c r="H38" s="38" t="inlineStr">
-        <is>
-          <t>~$0.5-1</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="42" t="inlineStr">
-        <is>
-          <t>Compass (Brookfield)</t>
-        </is>
-      </c>
-      <c r="B39" s="43" t="inlineStr">
-        <is>
-          <t>Undisclosed (Meta or MSFT)</t>
-        </is>
-      </c>
-      <c r="C39" s="43" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D39" s="43" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E39" s="54" t="inlineStr">
-        <is>
-          <t>Very High — single-tenant design</t>
-        </is>
-      </c>
-      <c r="F39" s="43" t="inlineStr">
-        <is>
-          <t>15-20</t>
-        </is>
-      </c>
-      <c r="G39" s="44" t="inlineStr">
-        <is>
-          <t>Single-tenant modular</t>
-        </is>
-      </c>
-      <c r="H39" s="43" t="inlineStr">
-        <is>
-          <t>~$1-2</t>
-        </is>
-      </c>
-      <c r="I39" s="52" t="n"/>
-      <c r="J39" s="52" t="n"/>
-    </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="10" t="inlineStr">
-        <is>
-          <t>Crusoe Energy</t>
-        </is>
-      </c>
-      <c r="B40" s="38" t="inlineStr">
-        <is>
-          <t>Oracle</t>
-        </is>
-      </c>
-      <c r="C40" s="38" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D40" s="38" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E40" s="55" t="inlineStr">
-        <is>
-          <t>Extreme — single customer</t>
-        </is>
-      </c>
-      <c r="F40" s="38" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="G40" s="41" t="inlineStr">
-        <is>
-          <t>Build-to-suit, triple-net</t>
-        </is>
-      </c>
-      <c r="H40" s="38" t="inlineStr">
-        <is>
-          <t>~$1-2</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="20" customHeight="1">
-      <c r="A41" s="42" t="inlineStr">
-        <is>
-          <t>Hut 8</t>
-        </is>
-      </c>
-      <c r="B41" s="43" t="inlineStr">
-        <is>
-          <t>Google (via Fluidstack)</t>
-        </is>
-      </c>
-      <c r="C41" s="43" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D41" s="43" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E41" s="55" t="inlineStr">
-        <is>
-          <t>Extreme — single customer</t>
-        </is>
-      </c>
-      <c r="F41" s="43" t="inlineStr">
-        <is>
-          <t>15 (+15 renewal)</t>
-        </is>
-      </c>
-      <c r="G41" s="44" t="inlineStr">
-        <is>
-          <t>Triple-net IT lease</t>
-        </is>
-      </c>
-      <c r="H41" s="43" t="inlineStr">
-        <is>
-          <t>~$0.5</t>
-        </is>
-      </c>
-      <c r="I41" s="52" t="n"/>
-      <c r="J41" s="52" t="n"/>
-    </row>
-    <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="10" t="inlineStr">
-        <is>
-          <t>Applied Digital</t>
-        </is>
-      </c>
-      <c r="B42" s="38" t="inlineStr">
-        <is>
-          <t>CoreWeave</t>
-        </is>
-      </c>
-      <c r="C42" s="38" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D42" s="38" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E42" s="55" t="inlineStr">
-        <is>
-          <t>Extreme — single customer</t>
-        </is>
-      </c>
-      <c r="F42" s="38" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="G42" s="41" t="inlineStr">
-        <is>
-          <t>Triple-net, GPU-ready</t>
-        </is>
-      </c>
-      <c r="H42" s="38" t="inlineStr">
-        <is>
-          <t>~$0.7</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="20" customHeight="1">
-      <c r="A43" s="42" t="inlineStr">
-        <is>
-          <t>EdgeConneX (EQT)</t>
-        </is>
-      </c>
-      <c r="B43" s="43" t="inlineStr">
-        <is>
-          <t>Mixed hyperscale + enterprise</t>
-        </is>
-      </c>
-      <c r="C43" s="43" t="inlineStr">
-        <is>
-          <t>Oracle</t>
-        </is>
-      </c>
-      <c r="D43" s="43" t="inlineStr">
-        <is>
-          <t>AWS / MSFT</t>
-        </is>
-      </c>
-      <c r="E43" s="44" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-      <c r="F43" s="43" t="inlineStr">
-        <is>
-          <t>10-15</t>
-        </is>
-      </c>
-      <c r="G43" s="44" t="inlineStr">
-        <is>
-          <t>Build-to-suit colo</t>
-        </is>
-      </c>
-      <c r="H43" s="43" t="inlineStr">
-        <is>
-          <t>~$0.5-1</t>
-        </is>
-      </c>
-      <c r="I43" s="52" t="n"/>
-      <c r="J43" s="52" t="n"/>
-    </row>
-    <row r="44" ht="20" customHeight="1"/>
-    <row r="45" ht="20" customHeight="1">
-      <c r="A45" s="15" t="inlineStr">
+      <c r="E52" s="53" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F52" s="59" t="inlineStr">
+        <is>
+          <t>5 yrs (compute)</t>
+        </is>
+      </c>
+      <c r="G52" s="61" t="inlineStr">
+        <is>
+          <t>GPU-aaS, take-or-pay</t>
+        </is>
+      </c>
+      <c r="H52" s="59" t="inlineStr">
+        <is>
+          <t>$3–5</t>
+        </is>
+      </c>
+      <c r="I52" s="61" t="inlineStr">
+        <is>
+          <t>Public (NASDAQ: CRWV). Nvidia-backed</t>
+        </is>
+      </c>
+      <c r="J52" s="64" t="n"/>
+      <c r="K52" s="64" t="n"/>
+    </row>
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="62" t="inlineStr">
+        <is>
+          <t>Nebius (NBIS)</t>
+        </is>
+      </c>
+      <c r="B53" s="59" t="inlineStr">
+        <is>
+          <t>Meta ($27B+$3B)</t>
+        </is>
+      </c>
+      <c r="C53" s="59" t="inlineStr">
+        <is>
+          <t>Microsoft (multi-B)</t>
+        </is>
+      </c>
+      <c r="D53" s="59" t="inlineStr">
+        <is>
+          <t>Enterprise / AI startups</t>
+        </is>
+      </c>
+      <c r="E53" s="54" t="inlineStr">
+        <is>
+          <t>Very High</t>
+        </is>
+      </c>
+      <c r="F53" s="59" t="inlineStr">
+        <is>
+          <t>5 yrs (infra delivery)</t>
+        </is>
+      </c>
+      <c r="G53" s="61" t="inlineStr">
+        <is>
+          <t>Full-stack AI cloud</t>
+        </is>
+      </c>
+      <c r="H53" s="59" t="inlineStr">
+        <is>
+          <t>$0.5–1</t>
+        </is>
+      </c>
+      <c r="I53" s="61" t="inlineStr">
+        <is>
+          <t>Public (NASDAQ: NBIS). Nvidia $2B</t>
+        </is>
+      </c>
+      <c r="J53" s="64" t="n"/>
+      <c r="K53" s="64" t="n"/>
+    </row>
+    <row r="54" ht="22" customHeight="1">
+      <c r="A54" s="62" t="inlineStr">
+        <is>
+          <t>IREN</t>
+        </is>
+      </c>
+      <c r="B54" s="59" t="inlineStr">
+        <is>
+          <t>Microsoft ($9.7B)</t>
+        </is>
+      </c>
+      <c r="C54" s="59" t="inlineStr">
+        <is>
+          <t>Together AI</t>
+        </is>
+      </c>
+      <c r="D54" s="59" t="inlineStr">
+        <is>
+          <t>Fluidstack / Fireworks AI</t>
+        </is>
+      </c>
+      <c r="E54" s="55" t="inlineStr">
+        <is>
+          <t>Extreme</t>
+        </is>
+      </c>
+      <c r="F54" s="59" t="inlineStr">
+        <is>
+          <t>5 yrs (MSFT)</t>
+        </is>
+      </c>
+      <c r="G54" s="61" t="inlineStr">
+        <is>
+          <t>GPU cloud + colocation</t>
+        </is>
+      </c>
+      <c r="H54" s="59" t="inlineStr">
+        <is>
+          <t>$1–2</t>
+        </is>
+      </c>
+      <c r="I54" s="61" t="inlineStr">
+        <is>
+          <t>Public (NASDAQ: IREN)</t>
+        </is>
+      </c>
+      <c r="J54" s="64" t="n"/>
+      <c r="K54" s="64" t="n"/>
+    </row>
+    <row r="55" ht="22" customHeight="1"/>
+    <row r="56" ht="22" customHeight="1">
+      <c r="A56" s="36" t="inlineStr">
+        <is>
+          <t>D. NEOCLOUD SUPPLY CHAIN: WHO THEY LEASE FROM → WHO THEY SELL TO</t>
+        </is>
+      </c>
+      <c r="B56" s="36" t="n"/>
+      <c r="C56" s="36" t="n"/>
+      <c r="D56" s="36" t="n"/>
+      <c r="E56" s="36" t="n"/>
+      <c r="F56" s="36" t="n"/>
+      <c r="G56" s="36" t="n"/>
+      <c r="H56" s="36" t="n"/>
+      <c r="I56" s="36" t="n"/>
+      <c r="J56" s="36" t="n"/>
+      <c r="K56" s="36" t="n"/>
+    </row>
+    <row r="57" ht="22" customHeight="1">
+      <c r="A57" s="45" t="inlineStr">
+        <is>
+          <t>Neocloud Provider</t>
+        </is>
+      </c>
+      <c r="B57" s="37" t="inlineStr">
+        <is>
+          <t>2025 Revenue ($B)</t>
+        </is>
+      </c>
+      <c r="C57" s="37" t="inlineStr">
+        <is>
+          <t>GPU Fleet</t>
+        </is>
+      </c>
+      <c r="D57" s="37" t="inlineStr">
+        <is>
+          <t>Leases DC Space From</t>
+        </is>
+      </c>
+      <c r="E57" s="37" t="inlineStr">
+        <is>
+          <t>Sells Compute To</t>
+        </is>
+      </c>
+      <c r="F57" s="37" t="inlineStr">
+        <is>
+          <t>Largest Contract ($B)</t>
+        </is>
+      </c>
+      <c r="G57" s="37" t="inlineStr">
+        <is>
+          <t>Nvidia Relationship</t>
+        </is>
+      </c>
+      <c r="H57" s="37" t="inlineStr">
+        <is>
+          <t>Capacity (MW)</t>
+        </is>
+      </c>
+      <c r="I57" s="37" t="inlineStr">
+        <is>
+          <t>2026E ARR Target ($B)</t>
+        </is>
+      </c>
+      <c r="J57" s="46" t="inlineStr"/>
+      <c r="K57" s="46" t="inlineStr"/>
+    </row>
+    <row r="58" ht="80" customHeight="1">
+      <c r="A58" s="58" t="inlineStr">
+        <is>
+          <t>CoreWeave (CRWV)</t>
+        </is>
+      </c>
+      <c r="B58" s="63" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="C58" s="59" t="inlineStr">
+        <is>
+          <t>250K+ GPUs</t>
+        </is>
+      </c>
+      <c r="D58" s="66" t="inlineStr">
+        <is>
+          <t>Applied Digital (400 MW)
+Core Scientific (1.3 GW, acquired)
+Digital Crossroads (180 MW)
+Chirisa (Lancaster PA, 300 MW)</t>
+        </is>
+      </c>
+      <c r="E58" s="66" t="inlineStr">
+        <is>
+          <t>OpenAI ($22.4B)
+Meta ($14.2B)
+Microsoft
+Google Cloud
+IBM</t>
+        </is>
+      </c>
+      <c r="F58" s="63" t="n">
+        <v>22.4</v>
+      </c>
+      <c r="G58" s="66" t="inlineStr">
+        <is>
+          <t>Largest customer (62% of 2024 rev). Guarantees leases. $6.3B compute backstop.</t>
+        </is>
+      </c>
+      <c r="H58" s="61" t="inlineStr">
+        <is>
+          <t>1,900</t>
+        </is>
+      </c>
+      <c r="I58" s="59" t="inlineStr">
+        <is>
+          <t>~10–12</t>
+        </is>
+      </c>
+      <c r="J58" s="64" t="n"/>
+      <c r="K58" s="64" t="n"/>
+    </row>
+    <row r="59" ht="80" customHeight="1">
+      <c r="A59" s="58" t="inlineStr">
+        <is>
+          <t>Nebius (NBIS)</t>
+        </is>
+      </c>
+      <c r="B59" s="63" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="C59" s="59" t="inlineStr">
+        <is>
+          <t>~30K+ GPUs</t>
+        </is>
+      </c>
+      <c r="D59" s="66" t="inlineStr">
+        <is>
+          <t>Patmos (Kansas City, colocation)
+Self-built: Vineland NJ (300 MW)
+Planned: Independence MO (800 MW)
+Mega Or (Israel, 80 MW)</t>
+        </is>
+      </c>
+      <c r="E59" s="66" t="inlineStr">
+        <is>
+          <t>Meta ($27B + $3B deals)
+Microsoft (multi-billion)
+AI startups &amp; enterprises</t>
+        </is>
+      </c>
+      <c r="F59" s="63" t="n">
+        <v>27</v>
+      </c>
+      <c r="G59" s="66" t="inlineStr">
+        <is>
+          <t>$2B strategic investment (Mar 2026). Full-stack partnership through Rubin platform.</t>
+        </is>
+      </c>
+      <c r="H59" s="61" t="inlineStr">
+        <is>
+          <t>170 (active)
+3,000+ (target end 2026)</t>
+        </is>
+      </c>
+      <c r="I59" s="59" t="inlineStr">
+        <is>
+          <t>7–9</t>
+        </is>
+      </c>
+      <c r="J59" s="64" t="n"/>
+      <c r="K59" s="64" t="n"/>
+    </row>
+    <row r="60" ht="80" customHeight="1">
+      <c r="A60" s="58" t="inlineStr">
+        <is>
+          <t>IREN</t>
+        </is>
+      </c>
+      <c r="B60" s="63" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="C60" s="59" t="inlineStr">
+        <is>
+          <t>~50K GPUs (target 150K)</t>
+        </is>
+      </c>
+      <c r="D60" s="66" t="inlineStr">
+        <is>
+          <t>Self-owned freehold sites:
+• Childress TX (750 MW)
+• Sweetwater TX
+• Mackenzie BC
+• Canal Flats BC</t>
+        </is>
+      </c>
+      <c r="E60" s="66" t="inlineStr">
+        <is>
+          <t>Microsoft ($9.7B / 5-yr)
+Together AI
+Fluidstack
+Fireworks AI
+Hume</t>
+        </is>
+      </c>
+      <c r="F60" s="63" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="G60" s="66" t="inlineStr">
+        <is>
+          <t>Purchases Nvidia B300 GPUs. Not equity-backed by Nvidia.</t>
+        </is>
+      </c>
+      <c r="H60" s="61" t="inlineStr">
+        <is>
+          <t>810 (operational)
+2,100 (under construction)</t>
+        </is>
+      </c>
+      <c r="I60" s="59" t="inlineStr">
+        <is>
+          <t>3.4–3.7</t>
+        </is>
+      </c>
+      <c r="J60" s="64" t="n"/>
+      <c r="K60" s="64" t="n"/>
+    </row>
+    <row r="61" ht="22" customHeight="1"/>
+    <row r="62" ht="22" customHeight="1">
+      <c r="A62" s="15" t="inlineStr">
         <is>
           <t>Sources &amp; Notes</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="16" t="inlineStr">
-        <is>
-          <t>Tenant relationships compiled from SEC filings, press releases, and industry reports (Q1 2026). Some relationships are inferred from public filings.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="20" customHeight="1">
-      <c r="A47" s="16" t="inlineStr">
-        <is>
-          <t>Oracle future lease commitments ($261B) per Oracle FY Q2 2026 10-Q. Microsoft ($155B) and Meta ($104B) per Bloomberg/company filings Mar 2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="20" customHeight="1">
-      <c r="A48" s="16" t="inlineStr">
-        <is>
-          <t>Moody's (Feb 2026): Big-5 hyperscalers hold $969B total undiscounted future lease commitments; $662B is off-balance-sheet (uncommenced).</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="20" customHeight="1">
-      <c r="A49" s="16" t="inlineStr">
-        <is>
-          <t>Crusoe → Oracle → Microsoft → OpenAI represents a multi-layered sublease chain; Stargate JV (Oracle/SoftBank/OpenAI) is a separate structure.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="20" customHeight="1">
-      <c r="A50" s="16" t="inlineStr">
-        <is>
-          <t>Meta increasingly uses SPV structures (Pimco debt + Blue Owl equity) for build-to-suit DCs, retaining 20% co-ownership while keeping lease off-balance-sheet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="20" customHeight="1">
-      <c r="A51" s="16" t="inlineStr">
-        <is>
-          <t>Revenue concentration risk ratings are editorial assessments; 'Extreme' = &gt;80% revenue from a single customer, 'Very High' = &gt;60% from top 2.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="20" customHeight="1">
-      <c r="A52" s="16" t="inlineStr">
-        <is>
-          <t>✓ = Confirmed tenant/customer relationship.  ~ = Suspected or indirect relationship.  Capacity figures are approximate operational + planned.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="20" customHeight="1">
-      <c r="A53" s="16" t="inlineStr">
-        <is>
-          <t>Amazon's total future lease commitments are not separately disclosed but estimated at $80-100B based on on-B/S liabilities and industry analysis.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="20" customHeight="1"/>
+    <row r="63" ht="22" customHeight="1">
+      <c r="A63" s="16" t="inlineStr">
+        <is>
+          <t>Tenant relationships compiled from SEC filings (10-K, 10-Q, S-1), press releases, and industry reports as of Q1 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="22" customHeight="1">
+      <c r="A64" s="16" t="inlineStr">
+        <is>
+          <t>Oracle future lease commitments ($261B) per 10-Q. Microsoft ($155B) and Meta ($104B) per Bloomberg/company filings Mar 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="22" customHeight="1">
+      <c r="A65" s="16" t="inlineStr">
+        <is>
+          <t>Moody's (Feb 2026): Big-5 hyperscalers hold $969B total undiscounted future lease commitments; $662B uncommenced (off-balance-sheet).</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="22" customHeight="1">
+      <c r="A66" s="16" t="inlineStr">
+        <is>
+          <t>CoreWeave RPO of $60.7B (Dec 2025 10-K). Revenue $5.1B (2025). Acquired Core Scientific for $9B (Jul 2025). IPO Mar 2025.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="22" customHeight="1">
+      <c r="A67" s="16" t="inlineStr">
+        <is>
+          <t>Nebius: Meta $27B deal (Mar 2026) + $3B deal (Nov 2025). Microsoft multi-B deal (Sep 2025). Nvidia $2B investment (Mar 2026). Revenue $530M (2025).</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="22" customHeight="1">
+      <c r="A68" s="16" t="inlineStr">
+        <is>
+          <t>IREN: Microsoft $9.7B/5-yr contract (Nov 2025). Revenue ~$960M annualized. Owns all sites freehold. Formerly Iris Energy. 150K GPU target by end 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="22" customHeight="1">
+      <c r="A69" s="16" t="inlineStr">
+        <is>
+          <t>Crusoe → Oracle → Microsoft → OpenAI is a multi-layered sublease chain; Stargate JV (Oracle/SoftBank/OpenAI) is a separate structure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="22" customHeight="1">
+      <c r="A70" s="16" t="inlineStr">
+        <is>
+          <t>✓ = Confirmed tenant/customer.  ~ = Suspected or indirect.  — = Self (not applicable).  Purple rows = neocloud providers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="22" customHeight="1">
+      <c r="A71" s="16" t="inlineStr">
+        <is>
+          <t>Concentration risk: Extreme (&gt;80% from 1 customer), Very High (&gt;60% from top 2), High (&gt;40% from top 2), Moderate, Low.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="22" customHeight="1"/>
   </sheetData>
-  <mergeCells count="13">
-    <mergeCell ref="A47:J47"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A46:J46"/>
-    <mergeCell ref="A22:J22"/>
-    <mergeCell ref="A30:J30"/>
-    <mergeCell ref="A53:J53"/>
-    <mergeCell ref="A50:J50"/>
-    <mergeCell ref="A4:J4"/>
-    <mergeCell ref="A48:J48"/>
-    <mergeCell ref="A51:J51"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A52:J52"/>
-    <mergeCell ref="A49:J49"/>
+  <mergeCells count="15">
+    <mergeCell ref="A70:K70"/>
+    <mergeCell ref="A69:K69"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A26:K26"/>
+    <mergeCell ref="A64:K64"/>
+    <mergeCell ref="A65:K65"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A63:K63"/>
+    <mergeCell ref="A71:K71"/>
+    <mergeCell ref="A68:K68"/>
+    <mergeCell ref="A66:K66"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A37:K37"/>
+    <mergeCell ref="A56:K56"/>
+    <mergeCell ref="A67:K67"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>